<commit_message>
Add reference answers and update Colab Ollama setup
</commit_message>
<xml_diff>
--- a/Questions.xlsx
+++ b/Questions.xlsx
@@ -449,61 +449,211 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA4C88A3-5EB2-49D0-AB22-0FEF6031D8A0}">
-  <dimension ref="A1:A10"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{DA4C88A3-5EB2-49D0-AB22-0FEF6031D8A0}">
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr defaultRowHeight="14.25" ns3:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="217.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:1" ns3:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>reference_answer</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>reference_source</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>reference_notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:1" ht="17.25" ns3:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>20 subjects will be recruited, specifically individuals living with spinal cord injury above C7.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>NCT06159946_Prot_000.pdf</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Verified from the study overview/sample description.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="17.25" ns3:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>The primary objective is to evaluate the feasibility of a co-designed, bespoke, high-immersion VR intervention for upper limb exercise during acute upper limb rehabilitation after spinal cord injury.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>NCT06154122_Prot_000.pdf</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Verified from the Study aims section, Primary Objective: Feasibility.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ns3:dyDescent="0.2">
       <c r="A4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>The MSC dressing is applied 4 times per day for 2 weeks.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>NCT06149832_Prot_000.pdf</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Verified from Treatment Protocol, Methods of stem cell administration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" spans="1:1" ht="17.25" ns3:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Emicizumab is administered subcutaneously.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>NCT06155955_Prot_SAP_000.pdf</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Verified from the study procedure dosing description for low-dose emicizumab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="17.25" ns3:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>The three control methods are voice, eye gaze, and machine vision. The two ADLs are drinking water and washing the face.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>NCT06159946_Prot_000.pdf</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Verified from Study Procedures describing Access-H2O control methods and ADL trials.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="17.25" ns3:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>The angular velocities are 60 degrees/second, 90 degrees/second, and 120 degrees/second. The golden indicator is peak torque, measured at 60 degrees/second.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>NCT06153992_Prot_SAP_000.pdf</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Verified from Materials and Methods and outcome assessment text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" spans="1:1" ht="17.25" ns3:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="9" spans="1:1" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Confidentiality is guarded by assigning subject IDs linked to names in a separate password-protected document accessible through a password-protected user account; physical documents are locked in a file cabinet in a locked office accessible only to the investigator. Documents are kept for two years before shredding.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>NCT06156735_Prot_SAP_000.pdf</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Verified from Safety Measurements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" spans="1:1" ht="17.25" ns3:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:1" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>The minimum sample size required per institution at a 95% confidence interval is 1,151. The assumed hypothetical frequency of the outcome factor is 50%.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>NCT06155006_Prot_SAP_000.pdf</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Verified from Sample size section and Table 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" spans="1:1" ht="17.25" ns3:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>The target sample size is 90 participants. The study originally required 41 participants per group, 82 total, and increased recruitment to 90 to account for an approximately 10% dropout rate.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>NCT06157684_Prot_000.pdf</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Verified from Sample size calculation.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add CSV file containing reference answers and update questions dataset
</commit_message>
<xml_diff>
--- a/Questions.xlsx
+++ b/Questions.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\talebi\Desktop\RAG Assignment\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alimollahosseini/Downloads/RAG Assignment/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9D36F1C0-0A01-4C5A-8543-06119BD7315A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{DD45CFC7-789D-6F49-BD75-235E61C044BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="27840" windowHeight="14220" xr2:uid="{945F73E5-75C0-47BE-BDEA-69C3098864D5}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="27840" windowHeight="14220" xr2:uid="{945F73E5-75C0-47BE-BDEA-69C3098864D5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="39">
   <si>
     <t>Questions</t>
   </si>
@@ -60,57 +61,110 @@
     <t>In the Music Therapy for cognition study (NCT06156735), how will subjects' confidentiality be guarded, and how long will documents be kept before shredding?</t>
   </si>
   <si>
-    <r>
-      <t>According to the Hepatitis C screening protocol (NCT06155006), what is the minimum sample size required </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="12"/>
-        <color rgb="FF0F1115"/>
-        <rFont val="Segoe UI"/>
-        <family val="2"/>
-      </rPr>
-      <t>per institution</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF0F1115"/>
-        <rFont val="Segoe UI"/>
-        <family val="2"/>
-      </rPr>
-      <t> with a 95% confidence interval, and what is the assumed hypothetical frequency of the outcome factor in the population?</t>
-    </r>
-  </si>
-  <si>
     <t>What is the total sample size targeted for the postprandial ambulation study in gestational diabetes (NCT06157684), and why was an extra ~10% added?</t>
+  </si>
+  <si>
+    <t>reference_answer</t>
+  </si>
+  <si>
+    <t>reference_source</t>
+  </si>
+  <si>
+    <t>reference_notes</t>
+  </si>
+  <si>
+    <t>20 subjects will be recruited, specifically individuals living with spinal cord injury above C7.</t>
+  </si>
+  <si>
+    <t>NCT06159946_Prot_000.pdf</t>
+  </si>
+  <si>
+    <t>Verified from the study overview/sample description.</t>
+  </si>
+  <si>
+    <t>The primary objective is to evaluate the feasibility of a co-designed, bespoke, high-immersion VR intervention for upper limb exercise during acute upper limb rehabilitation after spinal cord injury.</t>
+  </si>
+  <si>
+    <t>NCT06154122_Prot_000.pdf</t>
+  </si>
+  <si>
+    <t>Verified from the Study aims section, Primary Objective: Feasibility.</t>
+  </si>
+  <si>
+    <t>The MSC dressing is applied 4 times per day for 2 weeks.</t>
+  </si>
+  <si>
+    <t>NCT06149832_Prot_000.pdf</t>
+  </si>
+  <si>
+    <t>Verified from Treatment Protocol, Methods of stem cell administration.</t>
+  </si>
+  <si>
+    <t>Emicizumab is administered subcutaneously.</t>
+  </si>
+  <si>
+    <t>NCT06155955_Prot_SAP_000.pdf</t>
+  </si>
+  <si>
+    <t>Verified from the study procedure dosing description for low-dose emicizumab.</t>
+  </si>
+  <si>
+    <t>The three control methods are voice, eye gaze, and machine vision. The two ADLs are drinking water and washing the face.</t>
+  </si>
+  <si>
+    <t>Verified from Study Procedures describing Access-H2O control methods and ADL trials.</t>
+  </si>
+  <si>
+    <t>The angular velocities are 60 degrees/second, 90 degrees/second, and 120 degrees/second. The golden indicator is peak torque, measured at 60 degrees/second.</t>
+  </si>
+  <si>
+    <t>NCT06153992_Prot_SAP_000.pdf</t>
+  </si>
+  <si>
+    <t>Verified from Materials and Methods and outcome assessment text.</t>
+  </si>
+  <si>
+    <t>Confidentiality is guarded by assigning subject IDs linked to names in a separate password-protected document accessible through a password-protected user account; physical documents are locked in a file cabinet in a locked office accessible only to the investigator. Documents are kept for two years before shredding.</t>
+  </si>
+  <si>
+    <t>NCT06156735_Prot_SAP_000.pdf</t>
+  </si>
+  <si>
+    <t>Verified from Safety Measurements.</t>
+  </si>
+  <si>
+    <t>According to the Hepatitis C screening protocol (NCT06155006), what is the minimum sample size required per institution with a 95% confidence interval, and what is the assumed hypothetical frequency of the outcome factor in the population?</t>
+  </si>
+  <si>
+    <t>The minimum sample size required per institution at a 95% confidence interval is 1,151. The assumed hypothetical frequency of the outcome factor is 50%.</t>
+  </si>
+  <si>
+    <t>NCT06155006_Prot_SAP_000.pdf</t>
+  </si>
+  <si>
+    <t>Verified from Sample size section and Table 1.</t>
+  </si>
+  <si>
+    <t>The target sample size is 90 participants. The study originally required 41 participants per group, 82 total, and increased recruitment to 90 to account for an approximately 10% dropout rate.</t>
+  </si>
+  <si>
+    <t>NCT06157684_Prot_000.pdf</t>
+  </si>
+  <si>
+    <t>Verified from Sample size calculation.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF0F1115"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="12"/>
-      <color rgb="FF0F1115"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -133,9 +187,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -449,211 +502,154 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{DA4C88A3-5EB2-49D0-AB22-0FEF6031D8A0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultRowHeight="14.25" ns3:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="217.875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="188.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="245.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="67.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ns3:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>reference_answer</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>reference_source</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>reference_notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" spans="1:1" ht="17.25" ns3:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>20 subjects will be recruited, specifically individuals living with spinal cord injury above C7.</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>NCT06159946_Prot_000.pdf</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Verified from the study overview/sample description.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" spans="1:1" ht="17.25" ns3:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>The primary objective is to evaluate the feasibility of a co-designed, bespoke, high-immersion VR intervention for upper limb exercise during acute upper limb rehabilitation after spinal cord injury.</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>NCT06154122_Prot_000.pdf</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Verified from the Study aims section, Primary Objective: Feasibility.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" spans="1:1" ns3:dyDescent="0.2">
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>The MSC dressing is applied 4 times per day for 2 weeks.</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>NCT06149832_Prot_000.pdf</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Verified from Treatment Protocol, Methods of stem cell administration.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" spans="1:1" ht="17.25" ns3:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Emicizumab is administered subcutaneously.</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>NCT06155955_Prot_SAP_000.pdf</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Verified from the study procedure dosing description for low-dose emicizumab.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" spans="1:1" ht="17.25" ns3:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+      <c r="B5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>5</v>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>The three control methods are voice, eye gaze, and machine vision. The two ADLs are drinking water and washing the face.</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>NCT06159946_Prot_000.pdf</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Verified from Study Procedures describing Access-H2O control methods and ADL trials.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" spans="1:1" ht="17.25" ns3:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
+      <c r="B6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>6</v>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>The angular velocities are 60 degrees/second, 90 degrees/second, and 120 degrees/second. The golden indicator is peak torque, measured at 60 degrees/second.</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>NCT06153992_Prot_SAP_000.pdf</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Verified from Materials and Methods and outcome assessment text.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" spans="1:1" ht="17.25" ns3:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+      <c r="B7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>7</v>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Confidentiality is guarded by assigning subject IDs linked to names in a separate password-protected document accessible through a password-protected user account; physical documents are locked in a file cabinet in a locked office accessible only to the investigator. Documents are kept for two years before shredding.</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>NCT06156735_Prot_SAP_000.pdf</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Verified from Safety Measurements.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" spans="1:1" ht="17.25" ns3:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+      <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>8</v>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>The minimum sample size required per institution at a 95% confidence interval is 1,151. The assumed hypothetical frequency of the outcome factor is 50%.</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>NCT06155006_Prot_SAP_000.pdf</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Verified from Sample size section and Table 1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" spans="1:1" ht="17.25" ns3:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>The target sample size is 90 participants. The study originally required 41 participants per group, 82 total, and increased recruitment to 90 to account for an approximately 10% dropout rate.</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>NCT06157684_Prot_000.pdf</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Verified from Sample size calculation.</t>
-        </is>
+      <c r="B10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>